<commit_message>
moved or added result files
</commit_message>
<xml_diff>
--- a/results/spell/AEFGR/comparisons/lda/AEFGR-lda-comparison-sample2.xlsx
+++ b/results/spell/AEFGR/comparisons/lda/AEFGR-lda-comparison-sample2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kowk/Dropbox/Analysis/LDA-workshop/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kowk/Dropbox/GitHub/self-supervised-word-classification/results/spell/AEFGR/comparisons/lda/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{651201ED-05DF-9F46-8D42-BAB5650D37F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30345C0B-382D-CB4E-A480-FF292E3AB7CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10740" yWindow="740" windowWidth="27760" windowHeight="16940" activeTab="1" xr2:uid="{DEE78F81-9F55-1047-A14F-B31248FF1058}"/>
+    <workbookView xWindow="7060" yWindow="500" windowWidth="27760" windowHeight="16940" activeTab="1" xr2:uid="{DEE78F81-9F55-1047-A14F-B31248FF1058}"/>
   </bookViews>
   <sheets>
     <sheet name="0.99" sheetId="4" r:id="rId1"/>
@@ -234,6 +234,18 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
@@ -247,6 +259,66 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -380,78 +452,6 @@
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -503,16 +503,16 @@
     <tableColumn id="12" xr3:uid="{A61B2EF5-FD51-6046-B2F2-18D4DB6493E3}" name="term"/>
     <tableColumn id="10" xr3:uid="{4D708498-A357-324E-A4FB-DCAD32D7E984}" name="index"/>
     <tableColumn id="2" xr3:uid="{34200F0B-9DAE-314A-AA49-064DB8077316}" name="lang"/>
-    <tableColumn id="13" xr3:uid="{0E64B485-3735-0F4C-9C3F-401C187E8E59}" name="key" dataDxfId="26">
+    <tableColumn id="13" xr3:uid="{0E64B485-3735-0F4C-9C3F-401C187E8E59}" name="key" dataDxfId="22">
       <calculatedColumnFormula>CONCATENATE(Table1[[#This Row],[lang]],"-",Table1[[#This Row],[term]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{1B14066C-D440-144C-9DC7-BFC6943B760F}" name="3" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{CEEC403E-2613-D148-A306-580AAAA4EB8A}" name="4" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{243A6586-FE17-B24F-ADFD-B0605AE411BF}" name="5" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{4517DBBD-B2F7-B04E-92B6-E2C5586AA5F1}" name="6" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{50265DFE-3F3B-224C-8B6D-694D6D0EC0AD}" name="7" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{B93992B5-EDCB-7143-80BC-D6AF67A6A879}" name="10" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{758796C2-AE94-1549-ABEA-28EE5CBCF960}" name="15" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{1B14066C-D440-144C-9DC7-BFC6943B760F}" name="3" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{CEEC403E-2613-D148-A306-580AAAA4EB8A}" name="4" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{243A6586-FE17-B24F-ADFD-B0605AE411BF}" name="5" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{4517DBBD-B2F7-B04E-92B6-E2C5586AA5F1}" name="6" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{50265DFE-3F3B-224C-8B6D-694D6D0EC0AD}" name="7" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{B93992B5-EDCB-7143-80BC-D6AF67A6A879}" name="10" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{758796C2-AE94-1549-ABEA-28EE5CBCF960}" name="15" dataDxfId="15"/>
     <tableColumn id="11" xr3:uid="{15A6DEB7-FB79-BC44-8871-298FFE2933B0}" name="Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -533,13 +533,13 @@
     <tableColumn id="14" xr3:uid="{C0B17F37-B4FC-9D4B-9EAE-8066398C59EB}" name="key">
       <calculatedColumnFormula>CONCATENATE(Table13[[#This Row],[lang]],"-",Table13[[#This Row],[term]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E6374255-5660-E64B-A61E-3512827D8A94}" name="3" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{659000BB-0E22-5949-B62E-52138E3DF553}" name="4" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{78F49910-8C66-214B-92D6-C41A1B258E41}" name="5" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{F55E229D-D17B-3443-9DE6-C7B72CE1A728}" name="6" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{866D23A9-987D-6645-9E04-9C9D7A1FF775}" name="7" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{8828C2F7-7770-C641-B2A4-AB9185F9ECB7}" name="10" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{5C43A95D-8388-0548-BDAE-87CADDD7A522}" name="15" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{E6374255-5660-E64B-A61E-3512827D8A94}" name="3" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{659000BB-0E22-5949-B62E-52138E3DF553}" name="4" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{78F49910-8C66-214B-92D6-C41A1B258E41}" name="5" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{F55E229D-D17B-3443-9DE6-C7B72CE1A728}" name="6" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{866D23A9-987D-6645-9E04-9C9D7A1FF775}" name="7" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{8828C2F7-7770-C641-B2A4-AB9185F9ECB7}" name="10" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{5C43A95D-8388-0548-BDAE-87CADDD7A522}" name="15" dataDxfId="8"/>
     <tableColumn id="11" xr3:uid="{132BDAE0-575B-B044-9BAD-6E2A6C126094}" name="Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -553,28 +553,28 @@
     <tableColumn id="1" xr3:uid="{1BCE3F42-937D-E441-8141-353C7727D832}" name="term"/>
     <tableColumn id="2" xr3:uid="{DA4BA8D2-4F26-1643-B191-B95C5EC656BB}" name="index"/>
     <tableColumn id="3" xr3:uid="{11877A5E-E9F6-7443-B66E-00CA5E476CA9}" name="lang"/>
-    <tableColumn id="13" xr3:uid="{6FD83324-4DA8-3740-A993-B3B2287C6E78}" name="key" dataDxfId="11">
+    <tableColumn id="13" xr3:uid="{6FD83324-4DA8-3740-A993-B3B2287C6E78}" name="key" dataDxfId="7">
       <calculatedColumnFormula>CONCATENATE(Table3[[#This Row],[lang]],"-",Table3[[#This Row],[term]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{751388A7-2927-A844-9FB0-1A85DF4F82F6}" name="3" dataDxfId="10">
+    <tableColumn id="4" xr3:uid="{751388A7-2927-A844-9FB0-1A85DF4F82F6}" name="3" dataDxfId="6">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,F$2:F$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,F$30:F$54),(2*_xlpm.d*_xlpm.p)/(_xlpm.d+_xlpm.p))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{12205F21-2208-E741-8BE3-2F7FB738AC13}" name="4" dataDxfId="9">
+    <tableColumn id="5" xr3:uid="{12205F21-2208-E741-8BE3-2F7FB738AC13}" name="4" dataDxfId="5">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,G$2:G$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,G$30:G$54),(2*_xlpm.d*_xlpm.p)/(_xlpm.d+_xlpm.p))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0C25F879-88CA-0643-A213-8621BF657BB9}" name="5" dataDxfId="8">
+    <tableColumn id="6" xr3:uid="{0C25F879-88CA-0643-A213-8621BF657BB9}" name="5" dataDxfId="4">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,H$2:H$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,H$30:H$54),(2*_xlpm.d*_xlpm.p)/(_xlpm.d+_xlpm.p))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{41185E32-9305-1342-9CD0-890DD2C35EC6}" name="6" dataDxfId="7">
+    <tableColumn id="7" xr3:uid="{41185E32-9305-1342-9CD0-890DD2C35EC6}" name="6" dataDxfId="3">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,I$2:I$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,I$30:I$54),(2*_xlpm.d*_xlpm.p)/(_xlpm.d+_xlpm.p))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{1803148B-63EA-354A-B4B1-70EC64E34F90}" name="7" dataDxfId="6">
+    <tableColumn id="8" xr3:uid="{1803148B-63EA-354A-B4B1-70EC64E34F90}" name="7" dataDxfId="2">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,J$2:J$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,J$30:J$54),(2*_xlpm.d*_xlpm.p)/(_xlpm.d+_xlpm.p))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{AA704F6D-12C6-9E45-9F6D-466914BC2513}" name="10" dataDxfId="5">
+    <tableColumn id="9" xr3:uid="{AA704F6D-12C6-9E45-9F6D-466914BC2513}" name="10" dataDxfId="1">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,K$2:K$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,K$30:K$54),(2*_xlpm.d*_xlpm.p)/(_xlpm.d+_xlpm.p))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{45F5510B-3826-3C4C-ACE0-41105E749482}" name="15" dataDxfId="4">
+    <tableColumn id="10" xr3:uid="{45F5510B-3826-3C4C-ACE0-41105E749482}" name="15" dataDxfId="0">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,L$2:L$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,L$30:L$54),(2*_xlpm.d*_xlpm.p)/(_xlpm.d+_xlpm.p))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="11" xr3:uid="{1C0EBFD2-3E8F-FD41-A5FE-8A4F54EDCAB1}" name="Note"/>
@@ -664,14 +664,14 @@
     <tableColumn id="14" xr3:uid="{47742549-4FF7-8547-B6C2-F3C39F36D1E8}" name="key">
       <calculatedColumnFormula>CONCATENATE(Table15[[#This Row],[lang]],"-",Table15[[#This Row],[term]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{EB3B163F-570C-0142-BA9F-2F610124B8EF}" name="3" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{FCD0012F-63CC-C14E-BDDA-F1B7E4792C35}" name="4" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{227D0D55-6BD6-9D4F-93F1-D03C8A9DF0C5}" name="5" dataDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{6DFC86EA-93DD-F14E-8004-B72E0AF35216}" name="6" dataDxfId="43"/>
-    <tableColumn id="7" xr3:uid="{C9A3E6BA-55E6-8041-8731-CB5F5D9BDE1D}" name="7" dataDxfId="42"/>
-    <tableColumn id="8" xr3:uid="{23EB930C-F978-2046-BC01-9B1637D512C4}" name="10" dataDxfId="41"/>
-    <tableColumn id="13" xr3:uid="{C87864DF-5929-D94B-A9A3-4D20B1AB1549}" name="12" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{70CF0631-D89E-BE41-A6C2-CC5144752EF2}" name="15" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{EB3B163F-570C-0142-BA9F-2F610124B8EF}" name="3" dataDxfId="70"/>
+    <tableColumn id="4" xr3:uid="{FCD0012F-63CC-C14E-BDDA-F1B7E4792C35}" name="4" dataDxfId="69"/>
+    <tableColumn id="5" xr3:uid="{227D0D55-6BD6-9D4F-93F1-D03C8A9DF0C5}" name="5" dataDxfId="68"/>
+    <tableColumn id="6" xr3:uid="{6DFC86EA-93DD-F14E-8004-B72E0AF35216}" name="6" dataDxfId="67"/>
+    <tableColumn id="7" xr3:uid="{C9A3E6BA-55E6-8041-8731-CB5F5D9BDE1D}" name="7" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{23EB930C-F978-2046-BC01-9B1637D512C4}" name="10" dataDxfId="65"/>
+    <tableColumn id="13" xr3:uid="{C87864DF-5929-D94B-A9A3-4D20B1AB1549}" name="12" dataDxfId="64"/>
+    <tableColumn id="9" xr3:uid="{70CF0631-D89E-BE41-A6C2-CC5144752EF2}" name="15" dataDxfId="63"/>
     <tableColumn id="11" xr3:uid="{AD1CD97B-1116-4D49-BC8A-28B680490705}" name="Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -692,14 +692,14 @@
     <tableColumn id="14" xr3:uid="{E46D767B-C1D9-6C4A-BEAC-5090623DE1A9}" name="key">
       <calculatedColumnFormula>CONCATENATE(Table136[[#This Row],[lang]],"-",Table136[[#This Row],[term]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BF8EF8A8-8FB1-B34F-9648-9CDBADCD846D}" name="3" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{E0E78025-97F1-C94D-8B2E-ABDDCD894780}" name="4" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{0055F304-2C0A-D14E-BE16-57F92532C752}" name="5" dataDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{7F92559E-9738-7044-9646-80D1CBD6CF81}" name="6" dataDxfId="36"/>
-    <tableColumn id="7" xr3:uid="{E0C7CF31-989B-EA43-8024-1825BBB1FCE7}" name="7" dataDxfId="35"/>
-    <tableColumn id="8" xr3:uid="{0B4F2DCC-2001-3140-A1B9-5A8644C4C363}" name="10" dataDxfId="34"/>
-    <tableColumn id="13" xr3:uid="{A0AB5865-88BE-3A46-88C9-8B08A4C113D3}" name="12" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{B496A74C-C8EC-0040-90B7-22C0D35C974F}" name="15" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{BF8EF8A8-8FB1-B34F-9648-9CDBADCD846D}" name="3" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{E0E78025-97F1-C94D-8B2E-ABDDCD894780}" name="4" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{0055F304-2C0A-D14E-BE16-57F92532C752}" name="5" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{7F92559E-9738-7044-9646-80D1CBD6CF81}" name="6" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{E0C7CF31-989B-EA43-8024-1825BBB1FCE7}" name="7" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{0B4F2DCC-2001-3140-A1B9-5A8644C4C363}" name="10" dataDxfId="57"/>
+    <tableColumn id="13" xr3:uid="{A0AB5865-88BE-3A46-88C9-8B08A4C113D3}" name="12" dataDxfId="56"/>
+    <tableColumn id="9" xr3:uid="{B496A74C-C8EC-0040-90B7-22C0D35C974F}" name="15" dataDxfId="55"/>
     <tableColumn id="11" xr3:uid="{8A55AB5D-3545-844F-9AAF-D0191787A107}" name="Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -719,28 +719,28 @@
     <tableColumn id="13" xr3:uid="{2309C1F7-370B-8141-9612-1AEF2A46CFC0}" name="key">
       <calculatedColumnFormula>CONCATENATE(Table37[[#This Row],[lang]],"-",Table37[[#This Row],[term]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{4742B0DE-B2E1-CC45-9B2C-DF680F1F62A2}" name="3" dataDxfId="0">
+    <tableColumn id="4" xr3:uid="{4742B0DE-B2E1-CC45-9B2C-DF680F1F62A2}" name="3" dataDxfId="54">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,F$2:F$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,F$30:F$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{D6CCE6DD-07CC-F943-A5FF-28032C380FE7}" name="4" dataDxfId="32">
+    <tableColumn id="5" xr3:uid="{D6CCE6DD-07CC-F943-A5FF-28032C380FE7}" name="4" dataDxfId="53">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,G$2:G$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,G$30:G$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{FB9AF5D7-4603-724D-9070-781C5D60916C}" name="5" dataDxfId="31">
+    <tableColumn id="6" xr3:uid="{FB9AF5D7-4603-724D-9070-781C5D60916C}" name="5" dataDxfId="52">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,H$2:H$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,H$30:H$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{CDE845FF-C96D-B242-A17D-6F53BF08CFB0}" name="6" dataDxfId="30">
+    <tableColumn id="7" xr3:uid="{CDE845FF-C96D-B242-A17D-6F53BF08CFB0}" name="6" dataDxfId="51">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,I$2:I$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,I$30:I$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{31301EF2-DA57-CC4B-AA92-2FF70FCC99A6}" name="7" dataDxfId="29">
+    <tableColumn id="8" xr3:uid="{31301EF2-DA57-CC4B-AA92-2FF70FCC99A6}" name="7" dataDxfId="50">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,J$2:J$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,J$30:J$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{89C96574-69C4-7D47-B1D9-62D05FB66D31}" name="10" dataDxfId="28">
+    <tableColumn id="9" xr3:uid="{89C96574-69C4-7D47-B1D9-62D05FB66D31}" name="10" dataDxfId="49">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,K$2:K$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,K$30:K$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{606A8675-5F65-F54E-8FED-D32517E875F1}" name="12" dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{606A8675-5F65-F54E-8FED-D32517E875F1}" name="12" dataDxfId="48">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,L$2:L$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,L$30:L$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{7763F52B-0253-2D4F-81C8-CFED9CD14502}" name="15" dataDxfId="27">
+    <tableColumn id="10" xr3:uid="{7763F52B-0253-2D4F-81C8-CFED9CD14502}" name="15" dataDxfId="47">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,M$2:M$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,M$30:M$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="11" xr3:uid="{00028031-FFB8-244C-89AD-F41763B166E1}" name="Note"/>
@@ -760,16 +760,16 @@
     <tableColumn id="12" xr3:uid="{48C750D2-9EF8-5B43-B104-8E708E584A6B}" name="term"/>
     <tableColumn id="10" xr3:uid="{AFBC0544-BA49-9C48-9DD9-090C38028B4A}" name="index"/>
     <tableColumn id="2" xr3:uid="{54EE04F3-5F3E-A048-A408-7A4230219EFC}" name="lang"/>
-    <tableColumn id="13" xr3:uid="{4BC20366-49AB-3643-B374-4C6D839BED4C}" name="key" dataDxfId="70">
+    <tableColumn id="13" xr3:uid="{4BC20366-49AB-3643-B374-4C6D839BED4C}" name="key" dataDxfId="46">
       <calculatedColumnFormula>CONCATENATE(Table158[[#This Row],[lang]],"-",Table158[[#This Row],[term]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{62DC7C97-4EB2-194A-9581-4E26A79A0BEA}" name="3" dataDxfId="69"/>
-    <tableColumn id="4" xr3:uid="{970011EC-7AF1-EB4F-9A67-AB253B17F78C}" name="4" dataDxfId="68"/>
-    <tableColumn id="5" xr3:uid="{CEBAC408-E5E8-BF42-B313-00FBEA03F021}" name="5" dataDxfId="67"/>
-    <tableColumn id="6" xr3:uid="{6884CBAC-6DF6-3A45-A3C5-AAB67513F377}" name="6" dataDxfId="66"/>
-    <tableColumn id="7" xr3:uid="{857375B2-3C86-344B-AA8D-7F0239302FEA}" name="7" dataDxfId="65"/>
-    <tableColumn id="8" xr3:uid="{B16D5066-CA3F-C04D-8862-CCE5E41EACCF}" name="10" dataDxfId="64"/>
-    <tableColumn id="9" xr3:uid="{039AFE29-5E60-6E4B-AB7C-7EA46DD0F1A5}" name="15" dataDxfId="63"/>
+    <tableColumn id="3" xr3:uid="{62DC7C97-4EB2-194A-9581-4E26A79A0BEA}" name="3" dataDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{970011EC-7AF1-EB4F-9A67-AB253B17F78C}" name="4" dataDxfId="44"/>
+    <tableColumn id="5" xr3:uid="{CEBAC408-E5E8-BF42-B313-00FBEA03F021}" name="5" dataDxfId="43"/>
+    <tableColumn id="6" xr3:uid="{6884CBAC-6DF6-3A45-A3C5-AAB67513F377}" name="6" dataDxfId="42"/>
+    <tableColumn id="7" xr3:uid="{857375B2-3C86-344B-AA8D-7F0239302FEA}" name="7" dataDxfId="41"/>
+    <tableColumn id="8" xr3:uid="{B16D5066-CA3F-C04D-8862-CCE5E41EACCF}" name="10" dataDxfId="40"/>
+    <tableColumn id="9" xr3:uid="{039AFE29-5E60-6E4B-AB7C-7EA46DD0F1A5}" name="15" dataDxfId="39"/>
     <tableColumn id="11" xr3:uid="{D29D98BA-0801-9248-9319-2F44540464E0}" name="Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -787,16 +787,16 @@
     <tableColumn id="12" xr3:uid="{AE7CD974-A310-2849-A09F-06F4599E24EC}" name="term"/>
     <tableColumn id="10" xr3:uid="{54FF29EB-6A73-A34F-A4CF-AB2970998EAF}" name="index"/>
     <tableColumn id="2" xr3:uid="{A55B2DA9-F9CB-0844-9733-A48FE8AF39EC}" name="lang"/>
-    <tableColumn id="13" xr3:uid="{A2A6AE7D-EFB6-B246-9C02-4E4A543D9057}" name="key" dataDxfId="62">
+    <tableColumn id="13" xr3:uid="{A2A6AE7D-EFB6-B246-9C02-4E4A543D9057}" name="key" dataDxfId="38">
       <calculatedColumnFormula>CONCATENATE(Table1369[[#This Row],[lang]],"-",Table1369[[#This Row],[term]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{84D7BC35-F573-A74E-9328-4101147EF9D5}" name="3" dataDxfId="61"/>
-    <tableColumn id="4" xr3:uid="{68C2489F-D0EF-7F4D-B93E-7A3D0FCB4F0B}" name="4" dataDxfId="60"/>
-    <tableColumn id="5" xr3:uid="{9620607D-4A88-7F46-A120-EAD0AC33F342}" name="5" dataDxfId="59"/>
-    <tableColumn id="6" xr3:uid="{781D4B88-3EE6-C647-93AD-C29F21DAD3C5}" name="6" dataDxfId="58"/>
-    <tableColumn id="7" xr3:uid="{85B2AB5F-F5BE-354B-8FB3-821498D8BE5E}" name="7" dataDxfId="57"/>
-    <tableColumn id="8" xr3:uid="{BF04099E-C7FD-0341-8750-B49E2457AF18}" name="10" dataDxfId="56"/>
-    <tableColumn id="9" xr3:uid="{1001260D-A645-3749-A4A5-3C87AF86C058}" name="15" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{84D7BC35-F573-A74E-9328-4101147EF9D5}" name="3" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{68C2489F-D0EF-7F4D-B93E-7A3D0FCB4F0B}" name="4" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{9620607D-4A88-7F46-A120-EAD0AC33F342}" name="5" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{781D4B88-3EE6-C647-93AD-C29F21DAD3C5}" name="6" dataDxfId="34"/>
+    <tableColumn id="7" xr3:uid="{85B2AB5F-F5BE-354B-8FB3-821498D8BE5E}" name="7" dataDxfId="33"/>
+    <tableColumn id="8" xr3:uid="{BF04099E-C7FD-0341-8750-B49E2457AF18}" name="10" dataDxfId="32"/>
+    <tableColumn id="9" xr3:uid="{1001260D-A645-3749-A4A5-3C87AF86C058}" name="15" dataDxfId="31"/>
     <tableColumn id="11" xr3:uid="{BD48614D-C887-134F-B49E-8511A14FCC63}" name="Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -813,28 +813,28 @@
     <tableColumn id="1" xr3:uid="{D76EF8C3-EE7C-4A45-AF06-B2E184E3BF4C}" name="term"/>
     <tableColumn id="2" xr3:uid="{949599BA-78B0-2943-9CB2-2D90B394EF04}" name="index"/>
     <tableColumn id="3" xr3:uid="{CB98DFEF-76D1-4D42-96C0-FF839A68762F}" name="lang"/>
-    <tableColumn id="12" xr3:uid="{B5D9DC6E-2BBA-BF4F-B047-067D2615F4BB}" name="key" dataDxfId="54">
+    <tableColumn id="12" xr3:uid="{B5D9DC6E-2BBA-BF4F-B047-067D2615F4BB}" name="key" dataDxfId="30">
       <calculatedColumnFormula>CONCATENATE(Table3710[[#This Row],[lang]],"-",Table3710[[#This Row],[term]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{9FDDE5F0-59F3-EE4A-BF95-36417B52F8F0}" name="3" dataDxfId="53">
+    <tableColumn id="4" xr3:uid="{9FDDE5F0-59F3-EE4A-BF95-36417B52F8F0}" name="3" dataDxfId="29">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,F$2:F$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,F$30:F$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7C186066-287D-AC47-A92B-790569FE4EFC}" name="4" dataDxfId="52">
+    <tableColumn id="5" xr3:uid="{7C186066-287D-AC47-A92B-790569FE4EFC}" name="4" dataDxfId="28">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,G$2:G$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,G$30:G$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{771AF77C-E5ED-8E4E-89A4-AB40BC703B71}" name="5" dataDxfId="51">
+    <tableColumn id="6" xr3:uid="{771AF77C-E5ED-8E4E-89A4-AB40BC703B71}" name="5" dataDxfId="27">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,H$2:H$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,H$30:H$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{7377BC24-0AAB-D241-A95A-C2BCC39B18FE}" name="6" dataDxfId="50">
+    <tableColumn id="7" xr3:uid="{7377BC24-0AAB-D241-A95A-C2BCC39B18FE}" name="6" dataDxfId="26">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,I$2:I$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,I$30:I$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{242B5ACA-BBED-C142-8AAD-DEEF871F4BEA}" name="7" dataDxfId="49">
+    <tableColumn id="8" xr3:uid="{242B5ACA-BBED-C142-8AAD-DEEF871F4BEA}" name="7" dataDxfId="25">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,J$2:J$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,J$30:J$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{454139BE-6B64-CB40-AC02-1B553F3A1C88}" name="10" dataDxfId="48">
+    <tableColumn id="9" xr3:uid="{454139BE-6B64-CB40-AC02-1B553F3A1C88}" name="10" dataDxfId="24">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,K$2:K$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,K$30:K$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{08306E8D-62BA-414C-BA69-A71122A64717}" name="15" dataDxfId="47">
+    <tableColumn id="10" xr3:uid="{08306E8D-62BA-414C-BA69-A71122A64717}" name="15" dataDxfId="23">
       <calculatedColumnFormula>_xlfn.LET(_xlpm.r,$E58,_xlpm.d,_xlfn.XLOOKUP(_xlpm.r,$E$2:$E$26,L$2:L$26),_xlpm.p,_xlfn.XLOOKUP(_xlpm.r,$E$30:$E$54,L$30:L$54),IFERROR(2*_xlpm.d*_xlpm.p/(_xlpm.d+_xlpm.p),0))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="11" xr3:uid="{1F63154D-DE4B-904A-B9E8-5973D700C81D}" name="Note"/>
@@ -3663,7 +3663,7 @@
   <cols>
     <col min="1" max="1" width="8.625" customWidth="1"/>
     <col min="2" max="2" width="7.375" customWidth="1"/>
-    <col min="3" max="3" width="13.25" customWidth="1"/>
+    <col min="3" max="3" width="12.375" customWidth="1"/>
     <col min="4" max="4" width="9.625" customWidth="1"/>
     <col min="5" max="5" width="12.25" customWidth="1"/>
     <col min="6" max="13" width="7.625" customWidth="1"/>

</xml_diff>